<commit_message>
cambios sudoku sin C3
</commit_message>
<xml_diff>
--- a/SUDOKU.xlsx
+++ b/SUDOKU.xlsx
@@ -5,10 +5,10 @@
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gplaneta.sharepoint.com/sites/BIPOWER/Shared Documents/General/Distribución Atenea/Codigos/Distribución OBS/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\uscp9a\Distribución OBS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="478" documentId="13_ncr:1_{661915EF-FB0A-4BAE-BE12-09ADC5EFB6BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{03B4D355-D7DB-46E1-A0F8-9B1AF84E55BA}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AD06FF4-A909-423F-B378-69C0033412ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{EF95C2B5-218E-4516-887F-CDE11964293A}"/>
   </bookViews>
@@ -17,7 +17,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="100" r:id="rId2"/>
+    <pivotCache cacheId="268" r:id="rId2"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="23">
   <si>
     <t>SEM</t>
   </si>
@@ -69,9 +69,6 @@
   </si>
   <si>
     <t>C2</t>
-  </si>
-  <si>
-    <t>C3</t>
   </si>
   <si>
     <t>TL</t>
@@ -583,7 +580,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Oriol Larrea Vivés" refreshedDate="45958.509275810182" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="48" xr:uid="{93C581A5-61B5-40FF-AC76-618DD97B7B96}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Santiago Calvo Prieto" refreshedDate="45960.681586921295" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="48" xr:uid="{93C581A5-61B5-40FF-AC76-618DD97B7B96}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A2:C50" sheet="Estatus diario"/>
   </cacheSource>
@@ -606,17 +603,17 @@
         <s v="B2"/>
         <s v="C1"/>
         <s v="C2"/>
-        <s v="C3"/>
+        <m/>
         <s v="TL"/>
-        <m/>
         <s v="S2"/>
         <s v="S3"/>
         <s v="S4"/>
         <s v="S5"/>
+        <s v="C3" u="1"/>
       </sharedItems>
     </cacheField>
     <cacheField name="HS" numFmtId="0">
-      <sharedItems containsBlank="1" containsMixedTypes="1" containsNumber="1" containsInteger="1" minValue="0" maxValue="1872"/>
+      <sharedItems containsBlank="1" containsMixedTypes="1" containsNumber="1" containsInteger="1" minValue="0" maxValue="1662"/>
     </cacheField>
   </cacheFields>
   <extLst>
@@ -662,21 +659,21 @@
   <r>
     <x v="0"/>
     <x v="6"/>
-    <n v="210"/>
+    <m/>
   </r>
   <r>
     <x v="0"/>
     <x v="7"/>
-    <n v="1872"/>
+    <n v="1662"/>
   </r>
   <r>
     <x v="1"/>
+    <x v="6"/>
+    <m/>
+  </r>
+  <r>
+    <x v="2"/>
     <x v="8"/>
-    <m/>
-  </r>
-  <r>
-    <x v="2"/>
-    <x v="9"/>
     <s v="TL"/>
   </r>
   <r>
@@ -712,21 +709,21 @@
   <r>
     <x v="2"/>
     <x v="6"/>
-    <n v="214"/>
+    <m/>
   </r>
   <r>
     <x v="2"/>
     <x v="7"/>
-    <n v="1782"/>
+    <n v="1568"/>
   </r>
   <r>
     <x v="1"/>
-    <x v="8"/>
+    <x v="6"/>
     <m/>
   </r>
   <r>
     <x v="3"/>
-    <x v="10"/>
+    <x v="9"/>
     <s v="TL"/>
   </r>
   <r>
@@ -762,21 +759,21 @@
   <r>
     <x v="3"/>
     <x v="6"/>
-    <n v="224"/>
+    <m/>
   </r>
   <r>
     <x v="3"/>
     <x v="7"/>
-    <n v="1720"/>
+    <n v="1496"/>
   </r>
   <r>
     <x v="1"/>
-    <x v="8"/>
+    <x v="6"/>
     <m/>
   </r>
   <r>
     <x v="4"/>
-    <x v="11"/>
+    <x v="10"/>
     <s v="TL"/>
   </r>
   <r>
@@ -812,21 +809,21 @@
   <r>
     <x v="4"/>
     <x v="6"/>
-    <n v="54"/>
+    <m/>
   </r>
   <r>
     <x v="4"/>
     <x v="7"/>
-    <n v="383"/>
+    <n v="329"/>
   </r>
   <r>
     <x v="1"/>
-    <x v="8"/>
+    <x v="6"/>
     <m/>
   </r>
   <r>
     <x v="5"/>
-    <x v="12"/>
+    <x v="11"/>
     <s v="TL"/>
   </r>
   <r>
@@ -862,7 +859,7 @@
   <r>
     <x v="5"/>
     <x v="6"/>
-    <n v="0"/>
+    <m/>
   </r>
   <r>
     <x v="5"/>
@@ -873,8 +870,8 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{96476416-5E19-428A-9C28-862565FD05AB}" name="TablaDinámica2" cacheId="100" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="O9:W16" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{96476416-5E19-428A-9C28-862565FD05AB}" name="TablaDinámica2" cacheId="268" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="O10:V17" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="3">
     <pivotField axis="axisRow" showAll="0">
       <items count="7">
@@ -895,13 +892,13 @@
         <item x="3"/>
         <item x="4"/>
         <item x="5"/>
-        <item x="6"/>
+        <item m="1" x="12"/>
+        <item h="1" x="8"/>
         <item h="1" x="9"/>
         <item h="1" x="10"/>
         <item h="1" x="11"/>
-        <item h="1" x="12"/>
         <item h="1" x="7"/>
-        <item h="1" x="8"/>
+        <item h="1" x="6"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -933,7 +930,7 @@
   <colFields count="1">
     <field x="1"/>
   </colFields>
-  <colItems count="8">
+  <colItems count="7">
     <i>
       <x/>
     </i>
@@ -951,9 +948,6 @@
     </i>
     <i>
       <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
     </i>
     <i t="grand">
       <x/>
@@ -1300,20 +1294,20 @@
     <col min="14" max="14" width="5.5703125" customWidth="1"/>
     <col min="15" max="15" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="17" max="22" width="4" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="17" max="21" width="4" bestFit="1" customWidth="1"/>
+    <col min="22" max="23" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="24" max="26" width="3.140625" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="3" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="29" max="29" width="12.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A1" s="25" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="25" t="s">
         <v>20</v>
-      </c>
-      <c r="B1" s="25" t="s">
-        <v>21</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>2</v>
@@ -1326,7 +1320,7 @@
       <c r="I1" s="3"/>
       <c r="J1" s="3"/>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
@@ -1360,7 +1354,7 @@
       </c>
       <c r="J2" s="1"/>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>1</v>
       </c>
@@ -1392,7 +1386,7 @@
       </c>
       <c r="J3" s="3"/>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
         <v>1</v>
       </c>
@@ -1400,7 +1394,7 @@
         <v>5</v>
       </c>
       <c r="C4" s="11">
-        <f t="shared" ref="C4:C9" si="1">+SUM(D4:H4)</f>
+        <f t="shared" ref="C4:C8" si="1">+SUM(D4:H4)</f>
         <v>310</v>
       </c>
       <c r="D4">
@@ -1424,11 +1418,11 @@
       </c>
       <c r="J4" s="3"/>
       <c r="O4" s="31" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P4" s="31"/>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
         <v>1</v>
       </c>
@@ -1460,7 +1454,7 @@
       </c>
       <c r="J5" s="3"/>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
         <v>1</v>
       </c>
@@ -1492,7 +1486,7 @@
       </c>
       <c r="J6" s="3"/>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
         <v>1</v>
       </c>
@@ -1524,7 +1518,7 @@
       </c>
       <c r="J7" s="3"/>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
         <v>1</v>
       </c>
@@ -1556,109 +1550,59 @@
       </c>
       <c r="J8" s="3"/>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="B9" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="C9" s="11">
-        <f t="shared" si="1"/>
-        <v>210</v>
-      </c>
-      <c r="D9">
-        <v>42</v>
-      </c>
-      <c r="E9">
-        <v>42</v>
-      </c>
-      <c r="F9">
-        <v>42</v>
-      </c>
-      <c r="G9">
-        <v>42</v>
-      </c>
-      <c r="H9">
-        <v>42</v>
-      </c>
-      <c r="I9" s="26">
-        <f t="shared" si="2"/>
-        <v>7</v>
-      </c>
+      <c r="B9" s="15"/>
+      <c r="C9" s="11"/>
+      <c r="I9" s="26"/>
       <c r="J9" s="3"/>
-      <c r="O9" s="30" t="s">
-        <v>19</v>
-      </c>
-      <c r="P9" s="30" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
         <v>1</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C10" s="18">
         <f>SUM(C3:C9)</f>
-        <v>1872</v>
+        <v>1662</v>
       </c>
       <c r="D10" s="19">
         <f>SUM(D3:D9)</f>
-        <v>394</v>
+        <v>352</v>
       </c>
       <c r="E10" s="19">
         <f t="shared" ref="E10:H10" si="3">SUM(E3:E9)</f>
-        <v>388</v>
+        <v>346</v>
       </c>
       <c r="F10" s="19">
         <f t="shared" si="3"/>
-        <v>361</v>
+        <v>319</v>
       </c>
       <c r="G10" s="19">
         <f t="shared" si="3"/>
-        <v>358</v>
+        <v>316</v>
       </c>
       <c r="H10" s="19">
         <f t="shared" si="3"/>
-        <v>371</v>
+        <v>329</v>
       </c>
       <c r="I10" s="26">
         <f t="shared" si="2"/>
-        <v>62.4</v>
+        <v>55.4</v>
       </c>
       <c r="J10" s="20"/>
       <c r="O10" s="30" t="s">
-        <v>16</v>
-      </c>
-      <c r="P10" t="s">
-        <v>4</v>
-      </c>
-      <c r="Q10" t="s">
-        <v>5</v>
-      </c>
-      <c r="R10" t="s">
-        <v>6</v>
-      </c>
-      <c r="S10" t="s">
-        <v>7</v>
-      </c>
-      <c r="T10" t="s">
-        <v>8</v>
-      </c>
-      <c r="U10" t="s">
-        <v>9</v>
-      </c>
-      <c r="V10" t="s">
-        <v>10</v>
-      </c>
-      <c r="W10" t="s">
+        <v>18</v>
+      </c>
+      <c r="P10" s="30" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A11" s="5"/>
       <c r="B11" s="3"/>
       <c r="C11" s="2"/>
@@ -1669,43 +1613,40 @@
       <c r="H11" s="21"/>
       <c r="I11" s="3"/>
       <c r="J11" s="3"/>
-      <c r="O11" s="29" t="s">
-        <v>1</v>
-      </c>
-      <c r="P11" s="34">
-        <v>272</v>
-      </c>
-      <c r="Q11" s="34">
-        <v>310</v>
-      </c>
-      <c r="R11" s="34">
-        <v>305</v>
-      </c>
-      <c r="S11" s="34">
-        <v>273</v>
-      </c>
-      <c r="T11" s="34">
-        <v>232</v>
-      </c>
-      <c r="U11" s="34">
-        <v>270</v>
-      </c>
-      <c r="V11" s="34">
-        <v>210</v>
-      </c>
-      <c r="W11" s="34">
-        <v>1872</v>
-      </c>
-    </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="O11" s="30" t="s">
+        <v>15</v>
+      </c>
+      <c r="P11" t="s">
+        <v>4</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>5</v>
+      </c>
+      <c r="R11" t="s">
+        <v>6</v>
+      </c>
+      <c r="S11" t="s">
+        <v>7</v>
+      </c>
+      <c r="T11" t="s">
+        <v>8</v>
+      </c>
+      <c r="U11" t="s">
+        <v>9</v>
+      </c>
+      <c r="V11" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D12" s="8">
         <f>+H2+1</f>
@@ -1732,36 +1673,33 @@
       </c>
       <c r="J12" s="1"/>
       <c r="O12" s="29" t="s">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="P12" s="34">
+        <v>272</v>
+      </c>
+      <c r="Q12" s="34">
+        <v>310</v>
+      </c>
+      <c r="R12" s="34">
+        <v>305</v>
+      </c>
+      <c r="S12" s="34">
+        <v>273</v>
+      </c>
+      <c r="T12" s="34">
+        <v>232</v>
+      </c>
+      <c r="U12" s="34">
         <v>270</v>
       </c>
-      <c r="Q12" s="34">
-        <v>312</v>
-      </c>
-      <c r="R12" s="34">
-        <v>245</v>
-      </c>
-      <c r="S12" s="34">
-        <v>228</v>
-      </c>
-      <c r="T12" s="34">
-        <v>231</v>
-      </c>
-      <c r="U12" s="34">
-        <v>282</v>
-      </c>
       <c r="V12" s="34">
-        <v>214</v>
-      </c>
-      <c r="W12" s="34">
-        <v>1782</v>
-      </c>
-    </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
+        <v>1662</v>
+      </c>
+    </row>
+    <row r="13" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B13" s="10" t="s">
         <v>4</v>
@@ -1791,42 +1729,39 @@
       </c>
       <c r="J13" s="3"/>
       <c r="O13" s="29" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="P13" s="34">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="Q13" s="34">
-        <v>302</v>
+        <v>312</v>
       </c>
       <c r="R13" s="34">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="S13" s="34">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="T13" s="34">
-        <v>186</v>
+        <v>231</v>
       </c>
       <c r="U13" s="34">
-        <v>268</v>
+        <v>282</v>
       </c>
       <c r="V13" s="34">
-        <v>224</v>
-      </c>
-      <c r="W13" s="34">
-        <v>1720</v>
-      </c>
-    </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+        <v>1568</v>
+      </c>
+    </row>
+    <row r="14" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B14" s="14" t="s">
         <v>5</v>
       </c>
       <c r="C14" s="11">
-        <f t="shared" ref="C14:C19" si="5">+SUM(D14:H14)</f>
+        <f t="shared" ref="C14:C18" si="5">+SUM(D14:H14)</f>
         <v>312</v>
       </c>
       <c r="D14">
@@ -1850,36 +1785,33 @@
       </c>
       <c r="J14" s="3"/>
       <c r="O14" s="29" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="P14" s="34">
-        <v>54</v>
+        <v>267</v>
       </c>
       <c r="Q14" s="34">
-        <v>64</v>
+        <v>302</v>
       </c>
       <c r="R14" s="34">
-        <v>59</v>
+        <v>243</v>
       </c>
       <c r="S14" s="34">
-        <v>50</v>
+        <v>230</v>
       </c>
       <c r="T14" s="34">
-        <v>44</v>
+        <v>186</v>
       </c>
       <c r="U14" s="34">
-        <v>58</v>
+        <v>268</v>
       </c>
       <c r="V14" s="34">
-        <v>54</v>
-      </c>
-      <c r="W14" s="34">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+        <v>1496</v>
+      </c>
+    </row>
+    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B15" s="10" t="s">
         <v>6</v>
@@ -1909,36 +1841,33 @@
       </c>
       <c r="J15" s="3"/>
       <c r="O15" s="29" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="P15" s="34">
-        <v>0</v>
+        <v>54</v>
       </c>
       <c r="Q15" s="34">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="R15" s="34">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="S15" s="34">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="T15" s="34">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="U15" s="34">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="V15" s="34">
-        <v>0</v>
-      </c>
-      <c r="W15" s="34">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B16" s="14" t="s">
         <v>7</v>
@@ -1968,36 +1897,33 @@
       </c>
       <c r="J16" s="3"/>
       <c r="O16" s="29" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="P16" s="34">
-        <v>863</v>
+        <v>0</v>
       </c>
       <c r="Q16" s="34">
-        <v>988</v>
+        <v>0</v>
       </c>
       <c r="R16" s="34">
-        <v>852</v>
+        <v>0</v>
       </c>
       <c r="S16" s="34">
-        <v>781</v>
+        <v>0</v>
       </c>
       <c r="T16" s="34">
-        <v>693</v>
+        <v>0</v>
       </c>
       <c r="U16" s="34">
-        <v>878</v>
+        <v>0</v>
       </c>
       <c r="V16" s="34">
-        <v>702</v>
-      </c>
-      <c r="W16" s="34">
-        <v>5757</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B17" s="10" t="s">
         <v>8</v>
@@ -2026,10 +1952,34 @@
         <v>7.7</v>
       </c>
       <c r="J17" s="3"/>
+      <c r="O17" s="29" t="s">
+        <v>16</v>
+      </c>
+      <c r="P17" s="34">
+        <v>863</v>
+      </c>
+      <c r="Q17" s="34">
+        <v>988</v>
+      </c>
+      <c r="R17" s="34">
+        <v>852</v>
+      </c>
+      <c r="S17" s="34">
+        <v>781</v>
+      </c>
+      <c r="T17" s="34">
+        <v>693</v>
+      </c>
+      <c r="U17" s="34">
+        <v>878</v>
+      </c>
+      <c r="V17" s="34">
+        <v>5055</v>
+      </c>
     </row>
     <row r="18" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B18" s="10" t="s">
         <v>9</v>
@@ -2059,72 +2009,49 @@
       </c>
       <c r="J18" s="3"/>
     </row>
-    <row r="19" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:32" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="B19" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="C19" s="11">
-        <f t="shared" si="5"/>
-        <v>214</v>
-      </c>
-      <c r="D19">
-        <v>42</v>
-      </c>
-      <c r="E19">
-        <v>42</v>
-      </c>
-      <c r="F19">
-        <v>42</v>
-      </c>
-      <c r="G19">
-        <v>42</v>
-      </c>
-      <c r="H19">
-        <v>46</v>
-      </c>
-      <c r="I19" s="26">
-        <f t="shared" si="6"/>
-        <v>7.1333333333333329</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="B19" s="15"/>
+      <c r="C19" s="11"/>
+      <c r="I19" s="26"/>
       <c r="J19" s="3"/>
     </row>
     <row r="20" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B20" s="17" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C20" s="18">
         <f>SUM(C13:C19)</f>
-        <v>1782</v>
+        <v>1568</v>
       </c>
       <c r="D20" s="19">
         <f>SUM(D13:D19)</f>
-        <v>371</v>
+        <v>329</v>
       </c>
       <c r="E20" s="19">
         <f t="shared" ref="E20:H20" si="7">SUM(E13:E19)</f>
-        <v>372</v>
+        <v>330</v>
       </c>
       <c r="F20" s="19">
         <f t="shared" si="7"/>
-        <v>362</v>
+        <v>320</v>
       </c>
       <c r="G20" s="19">
         <f t="shared" si="7"/>
-        <v>318</v>
+        <v>276</v>
       </c>
       <c r="H20" s="19">
         <f t="shared" si="7"/>
-        <v>359</v>
+        <v>313</v>
       </c>
       <c r="I20" s="26">
         <f t="shared" si="6"/>
-        <v>59.4</v>
+        <v>52.266666666666666</v>
       </c>
       <c r="J20" s="20"/>
     </row>
@@ -2140,19 +2067,19 @@
       <c r="I21" s="3"/>
       <c r="J21" s="3"/>
       <c r="O21" s="31" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="P21" s="31"/>
     </row>
     <row r="22" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D22" s="8">
         <f>+H12+1</f>
@@ -2184,7 +2111,7 @@
     </row>
     <row r="23" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A23" s="13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B23" s="10" t="s">
         <v>4</v>
@@ -2216,13 +2143,13 @@
     </row>
     <row r="24" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A24" s="13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B24" s="14" t="s">
         <v>5</v>
       </c>
       <c r="C24" s="11">
-        <f t="shared" ref="C24:C29" si="9">+SUM(D24:H24)</f>
+        <f t="shared" ref="C24:C28" si="9">+SUM(D24:H24)</f>
         <v>302</v>
       </c>
       <c r="D24">
@@ -2248,7 +2175,7 @@
     </row>
     <row r="25" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A25" s="13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B25" s="10" t="s">
         <v>6</v>
@@ -2280,7 +2207,7 @@
     </row>
     <row r="26" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A26" s="13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B26" s="14" t="s">
         <v>7</v>
@@ -2312,7 +2239,7 @@
     </row>
     <row r="27" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A27" s="13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B27" s="10" t="s">
         <v>8</v>
@@ -2344,7 +2271,7 @@
     </row>
     <row r="28" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A28" s="13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B28" s="10" t="s">
         <v>9</v>
@@ -2374,72 +2301,49 @@
       </c>
       <c r="J28" s="3"/>
     </row>
-    <row r="29" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:32" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="B29" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="C29" s="11">
-        <f t="shared" si="9"/>
-        <v>224</v>
-      </c>
-      <c r="D29">
-        <v>40</v>
-      </c>
-      <c r="E29">
-        <v>46</v>
-      </c>
-      <c r="F29">
-        <v>46</v>
-      </c>
-      <c r="G29">
-        <v>46</v>
-      </c>
-      <c r="H29">
-        <v>46</v>
-      </c>
-      <c r="I29" s="26">
-        <f t="shared" si="10"/>
-        <v>7.4666666666666668</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="B29" s="15"/>
+      <c r="C29" s="11"/>
+      <c r="I29" s="26"/>
       <c r="J29" s="3"/>
     </row>
     <row r="30" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A30" s="13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B30" s="17" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C30" s="18">
-        <f>SUM(C23:C29)</f>
-        <v>1720</v>
+        <f t="shared" ref="C30:H30" si="11">SUM(C23:C29)</f>
+        <v>1496</v>
       </c>
       <c r="D30" s="19">
-        <f>SUM(D23:D29)</f>
-        <v>341</v>
+        <f t="shared" si="11"/>
+        <v>301</v>
       </c>
       <c r="E30" s="19">
-        <f t="shared" ref="E30:H30" si="11">SUM(E23:E29)</f>
-        <v>347</v>
+        <f t="shared" si="11"/>
+        <v>301</v>
       </c>
       <c r="F30" s="19">
         <f t="shared" si="11"/>
-        <v>347</v>
+        <v>301</v>
       </c>
       <c r="G30" s="19">
         <f t="shared" si="11"/>
-        <v>328</v>
+        <v>282</v>
       </c>
       <c r="H30" s="19">
         <f t="shared" si="11"/>
-        <v>357</v>
+        <v>311</v>
       </c>
       <c r="I30" s="26">
         <f t="shared" si="10"/>
-        <v>57.333333333333336</v>
+        <v>49.866666666666667</v>
       </c>
       <c r="J30" s="20"/>
     </row>
@@ -2458,13 +2362,13 @@
     </row>
     <row r="32" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D32" s="8">
         <f>+H22+1</f>
@@ -2494,7 +2398,7 @@
     </row>
     <row r="33" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A33" s="13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B33" s="10" t="s">
         <v>4</v>
@@ -2519,13 +2423,13 @@
     </row>
     <row r="34" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A34" s="13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B34" s="14" t="s">
         <v>5</v>
       </c>
       <c r="C34" s="11">
-        <f t="shared" ref="C34:C39" si="13">+SUM(D34:H34)</f>
+        <f t="shared" ref="C34:C38" si="13">+SUM(D34:H34)</f>
         <v>64</v>
       </c>
       <c r="D34" s="12">
@@ -2544,7 +2448,7 @@
     </row>
     <row r="35" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A35" s="13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B35" s="10" t="s">
         <v>6</v>
@@ -2569,7 +2473,7 @@
     </row>
     <row r="36" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A36" s="13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B36" s="14" t="s">
         <v>7</v>
@@ -2594,7 +2498,7 @@
     </row>
     <row r="37" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A37" s="13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B37" s="10" t="s">
         <v>8</v>
@@ -2619,7 +2523,7 @@
     </row>
     <row r="38" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A38" s="13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B38" s="10" t="s">
         <v>9</v>
@@ -2642,48 +2546,38 @@
       <c r="J38" s="3"/>
       <c r="AF38" s="27"/>
     </row>
-    <row r="39" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:32" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="B39" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="C39" s="11">
-        <f t="shared" si="13"/>
-        <v>54</v>
-      </c>
-      <c r="D39" s="16">
-        <v>54</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="B39" s="15"/>
+      <c r="C39" s="11"/>
+      <c r="D39" s="16"/>
       <c r="E39" s="16"/>
       <c r="F39" s="16"/>
       <c r="G39" s="16"/>
       <c r="H39" s="16"/>
-      <c r="I39" s="26">
-        <f t="shared" si="14"/>
-        <v>9</v>
-      </c>
+      <c r="I39" s="26"/>
       <c r="J39" s="3"/>
       <c r="AF39" s="27"/>
     </row>
     <row r="40" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A40" s="13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B40" s="17" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C40" s="18">
-        <f>SUM(C33:C39)</f>
-        <v>383</v>
+        <f t="shared" ref="C40:H40" si="15">SUM(C33:C39)</f>
+        <v>329</v>
       </c>
       <c r="D40" s="19">
-        <f>SUM(D33:D39)</f>
-        <v>383</v>
+        <f t="shared" si="15"/>
+        <v>329</v>
       </c>
       <c r="E40" s="19">
-        <f t="shared" ref="E40:H40" si="15">SUM(E33:E39)</f>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="F40" s="19">
@@ -2700,7 +2594,7 @@
       </c>
       <c r="I40" s="26">
         <f t="shared" si="14"/>
-        <v>12.766666666666667</v>
+        <v>10.966666666666667</v>
       </c>
       <c r="J40" s="20"/>
       <c r="AF40" s="27"/>
@@ -2720,13 +2614,13 @@
     </row>
     <row r="42" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D42" s="8">
         <f>+H32+1</f>
@@ -2756,7 +2650,7 @@
     </row>
     <row r="43" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A43" s="13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B43" s="10" t="s">
         <v>4</v>
@@ -2779,13 +2673,13 @@
     </row>
     <row r="44" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A44" s="13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B44" s="14" t="s">
         <v>5</v>
       </c>
       <c r="C44" s="11">
-        <f t="shared" ref="C44:C49" si="17">+SUM(D44:H44)</f>
+        <f t="shared" ref="C44:C48" si="17">+SUM(D44:H44)</f>
         <v>0</v>
       </c>
       <c r="D44" s="12"/>
@@ -2802,7 +2696,7 @@
     </row>
     <row r="45" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A45" s="13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B45" s="10" t="s">
         <v>6</v>
@@ -2825,7 +2719,7 @@
     </row>
     <row r="46" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A46" s="13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B46" s="14" t="s">
         <v>7</v>
@@ -2848,7 +2742,7 @@
     </row>
     <row r="47" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A47" s="13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B47" s="10" t="s">
         <v>8</v>
@@ -2871,7 +2765,7 @@
     </row>
     <row r="48" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A48" s="13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B48" s="10" t="s">
         <v>9</v>
@@ -2892,35 +2786,27 @@
       <c r="J48" s="3"/>
       <c r="AF48" s="27"/>
     </row>
-    <row r="49" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:32" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="B49" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="C49" s="11">
-        <f t="shared" si="17"/>
-        <v>0</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="B49" s="15"/>
+      <c r="C49" s="11"/>
       <c r="D49" s="16"/>
       <c r="E49" s="16"/>
       <c r="F49" s="16"/>
       <c r="G49" s="16"/>
       <c r="H49" s="16"/>
-      <c r="I49" s="26">
-        <f t="shared" si="18"/>
-        <v>0</v>
-      </c>
+      <c r="I49" s="26"/>
       <c r="J49" s="3"/>
       <c r="AF49" s="27"/>
     </row>
     <row r="50" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A50" s="13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B50" s="17" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C50" s="22">
         <f>SUM(C43:C49)</f>
@@ -3016,6 +2902,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="396b9688-3d64-4f4f-b40d-59fd809f50b1" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e4f8e1ef-7590-4615-a0b0-41d92864fb7e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -3024,7 +2921,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A62BD1A1B5CAC249A95BCCCA1576DD25" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ac690216a3feb446896882bf9e857d22">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e4f8e1ef-7590-4615-a0b0-41d92864fb7e" xmlns:ns3="396b9688-3d64-4f4f-b40d-59fd809f50b1" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fc1e276ee4a1c4eeb2be670671426ef6" ns2:_="" ns3:_="">
     <xsd:import namespace="e4f8e1ef-7590-4615-a0b0-41d92864fb7e"/>
@@ -3259,18 +3156,18 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="396b9688-3d64-4f4f-b40d-59fd809f50b1" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e4f8e1ef-7590-4615-a0b0-41d92864fb7e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{007506E0-0CDE-4051-B6C4-9C0A8A8B90A4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="396b9688-3d64-4f4f-b40d-59fd809f50b1"/>
+    <ds:schemaRef ds:uri="e4f8e1ef-7590-4615-a0b0-41d92864fb7e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{73BCA648-DFB0-4933-AD78-DBDD8CAF7C52}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -3278,7 +3175,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8039E8B4-6FF4-40F6-9FA1-E9DA9C439884}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3295,15 +3192,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{007506E0-0CDE-4051-B6C4-9C0A8A8B90A4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="396b9688-3d64-4f4f-b40d-59fd809f50b1"/>
-    <ds:schemaRef ds:uri="e4f8e1ef-7590-4615-a0b0-41d92864fb7e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Correciones filtros y app
</commit_message>
<xml_diff>
--- a/SUDOKU.xlsx
+++ b/SUDOKU.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gplaneta.sharepoint.com/sites/BIPOWER/Shared Documents/General/Distribución Atenea/Codigos/Distribución OBS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="363" documentId="13_ncr:1_{0AD06FF4-A909-423F-B378-69C0033412ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{417CE98F-DC79-4302-A893-B76A9B1BB777}"/>
+  <xr:revisionPtr revIDLastSave="364" documentId="13_ncr:1_{0AD06FF4-A909-423F-B378-69C0033412ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1F7E5DBE-A9BE-4103-BB1F-35FCC29679BB}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{EF95C2B5-218E-4516-887F-CDE11964293A}"/>
   </bookViews>
@@ -17,7 +17,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="274" r:id="rId2"/>
+    <pivotCache cacheId="0" r:id="rId2"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -1676,7 +1676,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{96476416-5E19-428A-9C28-862565FD05AB}" name="TablaDinámica2" cacheId="274" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{96476416-5E19-428A-9C28-862565FD05AB}" name="TablaDinámica2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="O10:V17" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="3">
     <pivotField axis="axisRow" showAll="0">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="J22" s="1"/>
       <c r="O22" s="28">
-        <v>46092.463194444441</v>
+        <v>46093.854166666664</v>
       </c>
     </row>
     <row r="23" spans="1:32">
@@ -3438,15 +3438,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="396b9688-3d64-4f4f-b40d-59fd809f50b1" xsi:nil="true"/>
@@ -3455,6 +3446,15 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3693,20 +3693,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{73BCA648-DFB0-4933-AD78-DBDD8CAF7C52}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{007506E0-0CDE-4051-B6C4-9C0A8A8B90A4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="396b9688-3d64-4f4f-b40d-59fd809f50b1"/>
     <ds:schemaRef ds:uri="e4f8e1ef-7590-4615-a0b0-41d92864fb7e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{73BCA648-DFB0-4933-AD78-DBDD8CAF7C52}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
cambios ingles - B2 100%
</commit_message>
<xml_diff>
--- a/SUDOKU.xlsx
+++ b/SUDOKU.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gplaneta.sharepoint.com/sites/BIPOWER/Shared Documents/General/Distribución Atenea/Codigos/Distribución OBS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="372" documentId="13_ncr:1_{0AD06FF4-A909-423F-B378-69C0033412ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{540BFB52-CF1C-459F-9A6C-ECEAE260F414}"/>
+  <xr:revisionPtr revIDLastSave="375" documentId="13_ncr:1_{0AD06FF4-A909-423F-B378-69C0033412ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{15E1D879-188C-41DC-84F1-50E29F7BEA75}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{EF95C2B5-218E-4516-887F-CDE11964293A}"/>
   </bookViews>
@@ -17,7 +17,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="17" r:id="rId2"/>
+    <pivotCache cacheId="1749" r:id="rId2"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -118,7 +118,7 @@
     <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="34">
+  <fonts count="34" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1155,14 +1155,12 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="304">
@@ -1485,7 +1483,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Santiago Calvo Prieto" refreshedDate="46127.481692824076" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="48" xr:uid="{93C581A5-61B5-40FF-AC76-618DD97B7B96}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Santiago Calvo Prieto" refreshedDate="46147.519752893517" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="48" xr:uid="{93C581A5-61B5-40FF-AC76-618DD97B7B96}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A2:C50" sheet="Estatus diario"/>
   </cacheSource>
@@ -1518,7 +1516,7 @@
       </sharedItems>
     </cacheField>
     <cacheField name="HS" numFmtId="0">
-      <sharedItems containsBlank="1" containsMixedTypes="1" containsNumber="1" containsInteger="1" minValue="0" maxValue="7402"/>
+      <sharedItems containsBlank="1" containsMixedTypes="1" containsNumber="1" containsInteger="1" minValue="0" maxValue="6798"/>
     </cacheField>
   </cacheFields>
   <extLst>
@@ -1534,32 +1532,32 @@
   <r>
     <x v="0"/>
     <x v="0"/>
-    <n v="1375"/>
+    <n v="1230"/>
   </r>
   <r>
     <x v="0"/>
     <x v="1"/>
-    <n v="1092"/>
+    <n v="1042"/>
   </r>
   <r>
     <x v="0"/>
     <x v="2"/>
-    <n v="1101"/>
+    <n v="1191"/>
   </r>
   <r>
     <x v="0"/>
     <x v="3"/>
-    <n v="1178"/>
+    <n v="1191"/>
   </r>
   <r>
     <x v="0"/>
     <x v="4"/>
-    <n v="1346"/>
+    <n v="1200"/>
   </r>
   <r>
     <x v="0"/>
     <x v="5"/>
-    <n v="1310"/>
+    <n v="944"/>
   </r>
   <r>
     <x v="0"/>
@@ -1569,7 +1567,7 @@
   <r>
     <x v="0"/>
     <x v="7"/>
-    <n v="7402"/>
+    <n v="6798"/>
   </r>
   <r>
     <x v="1"/>
@@ -1775,7 +1773,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{96476416-5E19-428A-9C28-862565FD05AB}" name="TablaDinámica2" cacheId="17" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{96476416-5E19-428A-9C28-862565FD05AB}" name="TablaDinámica2" cacheId="1749" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="O10:V17" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="3">
     <pivotField axis="axisRow" showAll="0">
@@ -2191,7 +2189,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC90F7AF-2A69-4C5E-9FF5-F9DB01805A13}">
   <dimension ref="A1:AF53"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="10" max="10" width="8" customWidth="1"/>
     <col min="11" max="11" width="7.85546875" customWidth="1"/>
@@ -2199,7 +2197,8 @@
     <col min="14" max="14" width="5.5703125" customWidth="1"/>
     <col min="15" max="15" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="17" max="21" width="5.140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="20" width="5.140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="4.140625" bestFit="1" customWidth="1"/>
     <col min="22" max="23" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="24" max="26" width="3.140625" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="3" bestFit="1" customWidth="1"/>
@@ -2207,7 +2206,7 @@
     <col min="29" max="29" width="12.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A1" s="25" t="s">
         <v>19</v>
       </c>
@@ -2225,7 +2224,7 @@
       <c r="I1" s="3"/>
       <c r="J1" s="3"/>
     </row>
-    <row r="2" spans="1:22">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
@@ -2236,30 +2235,30 @@
         <v>2</v>
       </c>
       <c r="D2" s="8">
-        <v>46084</v>
+        <v>46147</v>
       </c>
       <c r="E2" s="8">
         <f>+D2+1</f>
-        <v>46085</v>
+        <v>46148</v>
       </c>
       <c r="F2" s="8">
         <f t="shared" ref="F2:G2" si="0">+E2+1</f>
-        <v>46086</v>
+        <v>46149</v>
       </c>
       <c r="G2" s="8">
         <f t="shared" si="0"/>
-        <v>46087</v>
+        <v>46150</v>
       </c>
       <c r="H2" s="8">
         <f>+G2+3</f>
-        <v>46090</v>
+        <v>46153</v>
       </c>
       <c r="I2" s="9" t="s">
         <v>3</v>
       </c>
       <c r="J2" s="1"/>
     </row>
-    <row r="3" spans="1:22">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>1</v>
       </c>
@@ -2268,18 +2267,18 @@
       </c>
       <c r="C3" s="11">
         <f>+SUM(D3:H3)</f>
-        <v>1375</v>
-      </c>
-      <c r="D3" s="31">
-        <v>1375</v>
+        <v>1230</v>
+      </c>
+      <c r="D3" s="34">
+        <v>1230</v>
       </c>
       <c r="I3" s="26">
         <f>IFERROR(C3/6/COUNT(D3:H3),0)</f>
-        <v>229.16666666666666</v>
+        <v>205</v>
       </c>
       <c r="J3" s="3"/>
     </row>
-    <row r="4" spans="1:22">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
         <v>1</v>
       </c>
@@ -2288,22 +2287,22 @@
       </c>
       <c r="C4" s="11">
         <f t="shared" ref="C4:C8" si="1">+SUM(D4:H4)</f>
-        <v>1092</v>
-      </c>
-      <c r="D4" s="31">
-        <v>1092</v>
+        <v>1042</v>
+      </c>
+      <c r="D4" s="34">
+        <v>1042</v>
       </c>
       <c r="I4" s="26">
         <f t="shared" ref="I4:I10" si="2">IFERROR(C4/6/COUNT(D4:H4),0)</f>
-        <v>182</v>
+        <v>173.66666666666666</v>
       </c>
       <c r="J4" s="3"/>
-      <c r="O4" s="32" t="s">
+      <c r="O4" s="31" t="s">
         <v>21</v>
       </c>
-      <c r="P4" s="32"/>
-    </row>
-    <row r="5" spans="1:22">
+      <c r="P4" s="31"/>
+    </row>
+    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
         <v>1</v>
       </c>
@@ -2312,18 +2311,18 @@
       </c>
       <c r="C5" s="11">
         <f t="shared" si="1"/>
-        <v>1101</v>
-      </c>
-      <c r="D5" s="31">
-        <v>1101</v>
+        <v>1191</v>
+      </c>
+      <c r="D5" s="34">
+        <v>1191</v>
       </c>
       <c r="I5" s="26">
         <f t="shared" si="2"/>
-        <v>183.5</v>
+        <v>198.5</v>
       </c>
       <c r="J5" s="3"/>
     </row>
-    <row r="6" spans="1:22">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
         <v>1</v>
       </c>
@@ -2332,18 +2331,18 @@
       </c>
       <c r="C6" s="11">
         <f t="shared" si="1"/>
-        <v>1178</v>
-      </c>
-      <c r="D6" s="31">
-        <v>1178</v>
+        <v>1191</v>
+      </c>
+      <c r="D6" s="34">
+        <v>1191</v>
       </c>
       <c r="I6" s="26">
         <f t="shared" si="2"/>
-        <v>196.33333333333334</v>
+        <v>198.5</v>
       </c>
       <c r="J6" s="3"/>
     </row>
-    <row r="7" spans="1:22">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
         <v>1</v>
       </c>
@@ -2352,18 +2351,18 @@
       </c>
       <c r="C7" s="11">
         <f t="shared" si="1"/>
-        <v>1346</v>
-      </c>
-      <c r="D7" s="31">
-        <v>1346</v>
+        <v>1200</v>
+      </c>
+      <c r="D7" s="34">
+        <v>1200</v>
       </c>
       <c r="I7" s="26">
         <f t="shared" si="2"/>
-        <v>224.33333333333334</v>
+        <v>200</v>
       </c>
       <c r="J7" s="3"/>
     </row>
-    <row r="8" spans="1:22">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
         <v>1</v>
       </c>
@@ -2372,18 +2371,18 @@
       </c>
       <c r="C8" s="11">
         <f t="shared" si="1"/>
-        <v>1310</v>
-      </c>
-      <c r="D8" s="31">
-        <v>1310</v>
+        <v>944</v>
+      </c>
+      <c r="D8" s="34">
+        <v>944</v>
       </c>
       <c r="I8" s="26">
         <f t="shared" si="2"/>
-        <v>218.33333333333334</v>
+        <v>157.33333333333334</v>
       </c>
       <c r="J8" s="3"/>
     </row>
-    <row r="9" spans="1:22" hidden="1">
+    <row r="9" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
         <v>1</v>
       </c>
@@ -2392,7 +2391,7 @@
       <c r="I9" s="26"/>
       <c r="J9" s="3"/>
     </row>
-    <row r="10" spans="1:22">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
         <v>1</v>
       </c>
@@ -2401,11 +2400,11 @@
       </c>
       <c r="C10" s="18">
         <f>SUM(C3:C9)</f>
-        <v>7402</v>
+        <v>6798</v>
       </c>
       <c r="D10" s="19">
         <f>SUM(D3:D9)</f>
-        <v>7402</v>
+        <v>6798</v>
       </c>
       <c r="E10" s="19">
         <f t="shared" ref="E10:H10" si="3">SUM(E3:E9)</f>
@@ -2425,7 +2424,7 @@
       </c>
       <c r="I10" s="26">
         <f t="shared" si="2"/>
-        <v>246.73333333333335</v>
+        <v>226.6</v>
       </c>
       <c r="J10" s="20"/>
       <c r="O10" s="30" t="s">
@@ -2435,7 +2434,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:22">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A11" s="5"/>
       <c r="B11" s="3"/>
       <c r="C11" s="2"/>
@@ -2471,7 +2470,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:22">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>11</v>
       </c>
@@ -2483,23 +2482,23 @@
       </c>
       <c r="D12" s="8">
         <f>+H2+1</f>
-        <v>46091</v>
+        <v>46154</v>
       </c>
       <c r="E12" s="8">
         <f>+D12+1</f>
-        <v>46092</v>
+        <v>46155</v>
       </c>
       <c r="F12" s="8">
         <f t="shared" ref="F12:G12" si="4">+E12+1</f>
-        <v>46093</v>
+        <v>46156</v>
       </c>
       <c r="G12" s="8">
         <f t="shared" si="4"/>
-        <v>46094</v>
+        <v>46157</v>
       </c>
       <c r="H12" s="8">
         <f>+G12+3</f>
-        <v>46097</v>
+        <v>46160</v>
       </c>
       <c r="I12" s="9" t="s">
         <v>3</v>
@@ -2509,28 +2508,28 @@
         <v>1</v>
       </c>
       <c r="P12" s="35">
-        <v>1375</v>
+        <v>1230</v>
       </c>
       <c r="Q12" s="35">
-        <v>1092</v>
+        <v>1042</v>
       </c>
       <c r="R12" s="35">
-        <v>1101</v>
+        <v>1191</v>
       </c>
       <c r="S12" s="35">
-        <v>1178</v>
+        <v>1191</v>
       </c>
       <c r="T12" s="35">
-        <v>1346</v>
+        <v>1200</v>
       </c>
       <c r="U12" s="35">
-        <v>1310</v>
+        <v>944</v>
       </c>
       <c r="V12" s="35">
-        <v>7402</v>
-      </c>
-    </row>
-    <row r="13" spans="1:22">
+        <v>6798</v>
+      </c>
+    </row>
+    <row r="13" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
         <v>11</v>
       </c>
@@ -2571,7 +2570,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:22">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A14" s="13" t="s">
         <v>11</v>
       </c>
@@ -2612,7 +2611,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:22">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
         <v>11</v>
       </c>
@@ -2653,7 +2652,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:22">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
         <v>11</v>
       </c>
@@ -2694,7 +2693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:32">
+    <row r="17" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
         <v>11</v>
       </c>
@@ -2714,28 +2713,28 @@
         <v>16</v>
       </c>
       <c r="P17" s="35">
-        <v>1375</v>
+        <v>1230</v>
       </c>
       <c r="Q17" s="35">
-        <v>1092</v>
+        <v>1042</v>
       </c>
       <c r="R17" s="35">
-        <v>1101</v>
+        <v>1191</v>
       </c>
       <c r="S17" s="35">
-        <v>1178</v>
+        <v>1191</v>
       </c>
       <c r="T17" s="35">
-        <v>1346</v>
+        <v>1200</v>
       </c>
       <c r="U17" s="35">
-        <v>1310</v>
+        <v>944</v>
       </c>
       <c r="V17" s="35">
-        <v>7402</v>
-      </c>
-    </row>
-    <row r="18" spans="1:32">
+        <v>6798</v>
+      </c>
+    </row>
+    <row r="18" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
         <v>11</v>
       </c>
@@ -2752,7 +2751,7 @@
       </c>
       <c r="J18" s="3"/>
     </row>
-    <row r="19" spans="1:32" hidden="1">
+    <row r="19" spans="1:32" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="13" t="s">
         <v>11</v>
       </c>
@@ -2761,7 +2760,7 @@
       <c r="I19" s="26"/>
       <c r="J19" s="3"/>
     </row>
-    <row r="20" spans="1:32">
+    <row r="20" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A20" s="13" t="s">
         <v>11</v>
       </c>
@@ -2798,9 +2797,9 @@
       </c>
       <c r="J20" s="20"/>
     </row>
-    <row r="21" spans="1:32">
-      <c r="A21" s="33"/>
-      <c r="B21" s="33"/>
+    <row r="21" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A21" s="32"/>
+      <c r="B21" s="32"/>
       <c r="C21" s="2"/>
       <c r="D21" s="21"/>
       <c r="E21" s="21"/>
@@ -2809,12 +2808,12 @@
       <c r="H21" s="21"/>
       <c r="I21" s="3"/>
       <c r="J21" s="3"/>
-      <c r="O21" s="32" t="s">
+      <c r="O21" s="31" t="s">
         <v>22</v>
       </c>
-      <c r="P21" s="32"/>
-    </row>
-    <row r="22" spans="1:32">
+      <c r="P21" s="31"/>
+    </row>
+    <row r="22" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>12</v>
       </c>
@@ -2826,23 +2825,23 @@
       </c>
       <c r="D22" s="8">
         <f>+H12+1</f>
-        <v>46098</v>
+        <v>46161</v>
       </c>
       <c r="E22" s="8">
         <f>+D22+1</f>
-        <v>46099</v>
+        <v>46162</v>
       </c>
       <c r="F22" s="8">
         <f t="shared" ref="F22:G22" si="8">+E22+1</f>
-        <v>46100</v>
+        <v>46163</v>
       </c>
       <c r="G22" s="8">
         <f t="shared" si="8"/>
-        <v>46101</v>
+        <v>46164</v>
       </c>
       <c r="H22" s="8">
         <f>+G22+3</f>
-        <v>46104</v>
+        <v>46167</v>
       </c>
       <c r="I22" s="9" t="s">
         <v>3</v>
@@ -2852,7 +2851,7 @@
         <v>46112.854166666664</v>
       </c>
     </row>
-    <row r="23" spans="1:32">
+    <row r="23" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A23" s="13" t="s">
         <v>12</v>
       </c>
@@ -2869,7 +2868,7 @@
       </c>
       <c r="J23" s="3"/>
     </row>
-    <row r="24" spans="1:32">
+    <row r="24" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A24" s="13" t="s">
         <v>12</v>
       </c>
@@ -2886,7 +2885,7 @@
       </c>
       <c r="J24" s="3"/>
     </row>
-    <row r="25" spans="1:32">
+    <row r="25" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A25" s="13" t="s">
         <v>12</v>
       </c>
@@ -2903,7 +2902,7 @@
       </c>
       <c r="J25" s="3"/>
     </row>
-    <row r="26" spans="1:32">
+    <row r="26" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A26" s="13" t="s">
         <v>12</v>
       </c>
@@ -2920,7 +2919,7 @@
       </c>
       <c r="J26" s="3"/>
     </row>
-    <row r="27" spans="1:32">
+    <row r="27" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A27" s="13" t="s">
         <v>12</v>
       </c>
@@ -2937,7 +2936,7 @@
       </c>
       <c r="J27" s="3"/>
     </row>
-    <row r="28" spans="1:32">
+    <row r="28" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A28" s="13" t="s">
         <v>12</v>
       </c>
@@ -2954,7 +2953,7 @@
       </c>
       <c r="J28" s="3"/>
     </row>
-    <row r="29" spans="1:32" hidden="1">
+    <row r="29" spans="1:32" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="13" t="s">
         <v>12</v>
       </c>
@@ -2963,7 +2962,7 @@
       <c r="I29" s="26"/>
       <c r="J29" s="3"/>
     </row>
-    <row r="30" spans="1:32">
+    <row r="30" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A30" s="13" t="s">
         <v>12</v>
       </c>
@@ -3000,9 +2999,9 @@
       </c>
       <c r="J30" s="20"/>
     </row>
-    <row r="31" spans="1:32">
-      <c r="A31" s="34"/>
-      <c r="B31" s="34"/>
+    <row r="31" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A31" s="33"/>
+      <c r="B31" s="33"/>
       <c r="C31" s="3"/>
       <c r="D31" s="3"/>
       <c r="E31" s="3"/>
@@ -3013,7 +3012,7 @@
       <c r="J31" s="3"/>
       <c r="AF31" s="27"/>
     </row>
-    <row r="32" spans="1:32">
+    <row r="32" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
         <v>13</v>
       </c>
@@ -3025,23 +3024,23 @@
       </c>
       <c r="D32" s="8">
         <f>+H22+1</f>
-        <v>46105</v>
+        <v>46168</v>
       </c>
       <c r="E32" s="8">
         <f>+D32+1</f>
-        <v>46106</v>
+        <v>46169</v>
       </c>
       <c r="F32" s="8">
         <f t="shared" ref="F32:G32" si="12">+E32+1</f>
-        <v>46107</v>
+        <v>46170</v>
       </c>
       <c r="G32" s="8">
         <f t="shared" si="12"/>
-        <v>46108</v>
+        <v>46171</v>
       </c>
       <c r="H32" s="8">
         <f>+G32+3</f>
-        <v>46111</v>
+        <v>46174</v>
       </c>
       <c r="I32" s="9" t="s">
         <v>3</v>
@@ -3049,7 +3048,7 @@
       <c r="J32" s="1"/>
       <c r="AF32" s="27"/>
     </row>
-    <row r="33" spans="1:32">
+    <row r="33" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A33" s="13" t="s">
         <v>13</v>
       </c>
@@ -3071,7 +3070,7 @@
       <c r="J33" s="3"/>
       <c r="AF33" s="27"/>
     </row>
-    <row r="34" spans="1:32">
+    <row r="34" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A34" s="13" t="s">
         <v>13</v>
       </c>
@@ -3093,7 +3092,7 @@
       <c r="J34" s="3"/>
       <c r="AF34" s="27"/>
     </row>
-    <row r="35" spans="1:32">
+    <row r="35" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A35" s="13" t="s">
         <v>13</v>
       </c>
@@ -3115,7 +3114,7 @@
       <c r="J35" s="3"/>
       <c r="AF35" s="27"/>
     </row>
-    <row r="36" spans="1:32">
+    <row r="36" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A36" s="13" t="s">
         <v>13</v>
       </c>
@@ -3137,7 +3136,7 @@
       <c r="J36" s="3"/>
       <c r="AF36" s="27"/>
     </row>
-    <row r="37" spans="1:32">
+    <row r="37" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A37" s="13" t="s">
         <v>13</v>
       </c>
@@ -3159,7 +3158,7 @@
       <c r="J37" s="3"/>
       <c r="AF37" s="27"/>
     </row>
-    <row r="38" spans="1:32">
+    <row r="38" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A38" s="13" t="s">
         <v>13</v>
       </c>
@@ -3181,7 +3180,7 @@
       <c r="J38" s="3"/>
       <c r="AF38" s="27"/>
     </row>
-    <row r="39" spans="1:32" hidden="1">
+    <row r="39" spans="1:32" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="13" t="s">
         <v>13</v>
       </c>
@@ -3196,7 +3195,7 @@
       <c r="J39" s="3"/>
       <c r="AF39" s="27"/>
     </row>
-    <row r="40" spans="1:32">
+    <row r="40" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A40" s="13" t="s">
         <v>13</v>
       </c>
@@ -3234,9 +3233,9 @@
       <c r="J40" s="20"/>
       <c r="AF40" s="27"/>
     </row>
-    <row r="41" spans="1:32">
-      <c r="A41" s="34"/>
-      <c r="B41" s="34"/>
+    <row r="41" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A41" s="33"/>
+      <c r="B41" s="33"/>
       <c r="C41" s="3"/>
       <c r="D41" s="3"/>
       <c r="E41" s="3"/>
@@ -3247,7 +3246,7 @@
       <c r="J41" s="3"/>
       <c r="AF41" s="27"/>
     </row>
-    <row r="42" spans="1:32">
+    <row r="42" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
         <v>14</v>
       </c>
@@ -3259,23 +3258,23 @@
       </c>
       <c r="D42" s="8">
         <f>+H32+1</f>
-        <v>46112</v>
+        <v>46175</v>
       </c>
       <c r="E42" s="8">
         <f>+D42+1</f>
-        <v>46113</v>
+        <v>46176</v>
       </c>
       <c r="F42" s="8">
         <f t="shared" ref="F42:G42" si="16">+E42+1</f>
-        <v>46114</v>
+        <v>46177</v>
       </c>
       <c r="G42" s="8">
         <f t="shared" si="16"/>
-        <v>46115</v>
+        <v>46178</v>
       </c>
       <c r="H42" s="8">
         <f>+G42+3</f>
-        <v>46118</v>
+        <v>46181</v>
       </c>
       <c r="I42" s="9" t="s">
         <v>3</v>
@@ -3283,7 +3282,7 @@
       <c r="J42" s="1"/>
       <c r="AF42" s="27"/>
     </row>
-    <row r="43" spans="1:32">
+    <row r="43" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A43" s="13" t="s">
         <v>14</v>
       </c>
@@ -3306,7 +3305,7 @@
       <c r="J43" s="3"/>
       <c r="AF43" s="27"/>
     </row>
-    <row r="44" spans="1:32">
+    <row r="44" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A44" s="13" t="s">
         <v>14</v>
       </c>
@@ -3329,7 +3328,7 @@
       <c r="J44" s="3"/>
       <c r="AF44" s="27"/>
     </row>
-    <row r="45" spans="1:32">
+    <row r="45" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A45" s="13" t="s">
         <v>14</v>
       </c>
@@ -3352,7 +3351,7 @@
       <c r="J45" s="3"/>
       <c r="AF45" s="27"/>
     </row>
-    <row r="46" spans="1:32">
+    <row r="46" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A46" s="13" t="s">
         <v>14</v>
       </c>
@@ -3375,7 +3374,7 @@
       <c r="J46" s="3"/>
       <c r="AF46" s="27"/>
     </row>
-    <row r="47" spans="1:32">
+    <row r="47" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A47" s="13" t="s">
         <v>14</v>
       </c>
@@ -3398,7 +3397,7 @@
       <c r="J47" s="3"/>
       <c r="AF47" s="27"/>
     </row>
-    <row r="48" spans="1:32">
+    <row r="48" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A48" s="13" t="s">
         <v>14</v>
       </c>
@@ -3421,7 +3420,7 @@
       <c r="J48" s="3"/>
       <c r="AF48" s="27"/>
     </row>
-    <row r="49" spans="1:32" hidden="1">
+    <row r="49" spans="1:32" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="13" t="s">
         <v>14</v>
       </c>
@@ -3436,7 +3435,7 @@
       <c r="J49" s="3"/>
       <c r="AF49" s="27"/>
     </row>
-    <row r="50" spans="1:32">
+    <row r="50" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A50" s="13" t="s">
         <v>14</v>
       </c>
@@ -3474,9 +3473,9 @@
       <c r="J50" s="20"/>
       <c r="AF50" s="27"/>
     </row>
-    <row r="51" spans="1:32">
-      <c r="A51" s="33"/>
-      <c r="B51" s="33"/>
+    <row r="51" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A51" s="32"/>
+      <c r="B51" s="32"/>
       <c r="C51" s="2"/>
       <c r="D51" s="24"/>
       <c r="E51" s="24"/>
@@ -3487,9 +3486,9 @@
       <c r="J51" s="3"/>
       <c r="AF51" s="27"/>
     </row>
-    <row r="52" spans="1:32">
-      <c r="A52" s="33"/>
-      <c r="B52" s="33"/>
+    <row r="52" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A52" s="32"/>
+      <c r="B52" s="32"/>
       <c r="C52" s="2"/>
       <c r="D52" s="21">
         <v>0</v>
@@ -3509,9 +3508,9 @@
       <c r="I52" s="3"/>
       <c r="J52" s="3"/>
     </row>
-    <row r="53" spans="1:32">
-      <c r="A53" s="33"/>
-      <c r="B53" s="33"/>
+    <row r="53" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="A53" s="32"/>
+      <c r="B53" s="32"/>
       <c r="C53" s="3"/>
       <c r="D53" s="3"/>
       <c r="E53" s="3"/>
@@ -3548,15 +3547,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A62BD1A1B5CAC249A95BCCCA1576DD25" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="95d80e3e9b41a0cd0f31651385762a39">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e4f8e1ef-7590-4615-a0b0-41d92864fb7e" xmlns:ns3="396b9688-3d64-4f4f-b40d-59fd809f50b1" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0c785e827d86c3245c0f7c251e0c72c1" ns2:_="" ns3:_="">
     <xsd:import namespace="e4f8e1ef-7590-4615-a0b0-41d92864fb7e"/>
@@ -3791,6 +3781,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{007506E0-0CDE-4051-B6C4-9C0A8A8B90A4}">
   <ds:schemaRefs>
@@ -3803,14 +3802,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{73BCA648-DFB0-4933-AD78-DBDD8CAF7C52}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{36A93179-9D9C-4D14-A08B-C1A220B5EC1D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3827,4 +3818,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{73BCA648-DFB0-4933-AD78-DBDD8CAF7C52}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
correciones finales 7 equipos
</commit_message>
<xml_diff>
--- a/SUDOKU.xlsx
+++ b/SUDOKU.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gplaneta.sharepoint.com/sites/BIPOWER/Shared Documents/General/Distribución Atenea/Codigos/Distribución OBS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="378" documentId="13_ncr:1_{0AD06FF4-A909-423F-B378-69C0033412ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{96B22DE9-845C-4012-9719-3BCEAAC603ED}"/>
+  <xr:revisionPtr revIDLastSave="382" documentId="13_ncr:1_{0AD06FF4-A909-423F-B378-69C0033412ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D37F5BCD-5942-498E-BE59-0F1DF6A5CC1F}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-45" windowWidth="29040" windowHeight="15720" xr2:uid="{EF95C2B5-218E-4516-887F-CDE11964293A}"/>
   </bookViews>
@@ -17,7 +17,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="139" r:id="rId2"/>
+    <pivotCache cacheId="790" r:id="rId2"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -1155,14 +1155,12 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="304">
@@ -1485,7 +1483,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Santiago Calvo Prieto" refreshedDate="46148.494425810182" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="48" xr:uid="{93C581A5-61B5-40FF-AC76-618DD97B7B96}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Santiago Calvo Prieto" refreshedDate="46148.707666087961" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="48" xr:uid="{93C581A5-61B5-40FF-AC76-618DD97B7B96}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A2:C50" sheet="Estatus diario"/>
   </cacheSource>
@@ -1518,7 +1516,7 @@
       </sharedItems>
     </cacheField>
     <cacheField name="HS" numFmtId="0">
-      <sharedItems containsBlank="1" containsMixedTypes="1" containsNumber="1" containsInteger="1" minValue="0" maxValue="7402"/>
+      <sharedItems containsBlank="1" containsMixedTypes="1" containsNumber="1" containsInteger="1" minValue="0" maxValue="6798"/>
     </cacheField>
   </cacheFields>
   <extLst>
@@ -1534,32 +1532,32 @@
   <r>
     <x v="0"/>
     <x v="0"/>
-    <n v="1375"/>
+    <n v="1230"/>
   </r>
   <r>
     <x v="0"/>
     <x v="1"/>
-    <n v="1092"/>
+    <n v="1042"/>
   </r>
   <r>
     <x v="0"/>
     <x v="2"/>
-    <n v="1101"/>
+    <n v="1191"/>
   </r>
   <r>
     <x v="0"/>
     <x v="3"/>
-    <n v="1178"/>
+    <n v="1191"/>
   </r>
   <r>
     <x v="0"/>
     <x v="4"/>
-    <n v="1346"/>
+    <n v="1200"/>
   </r>
   <r>
     <x v="0"/>
     <x v="5"/>
-    <n v="1310"/>
+    <n v="944"/>
   </r>
   <r>
     <x v="0"/>
@@ -1569,7 +1567,7 @@
   <r>
     <x v="0"/>
     <x v="7"/>
-    <n v="7402"/>
+    <n v="6798"/>
   </r>
   <r>
     <x v="1"/>
@@ -1775,7 +1773,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{96476416-5E19-428A-9C28-862565FD05AB}" name="TablaDinámica2" cacheId="139" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{96476416-5E19-428A-9C28-862565FD05AB}" name="TablaDinámica2" cacheId="790" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="O10:V17" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="3">
     <pivotField axis="axisRow" showAll="0">
@@ -2199,7 +2197,8 @@
     <col min="14" max="14" width="5.5703125" customWidth="1"/>
     <col min="15" max="15" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="17" max="21" width="5.140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="20" width="5.140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="4.140625" bestFit="1" customWidth="1"/>
     <col min="22" max="23" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="24" max="26" width="3.140625" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="3" bestFit="1" customWidth="1"/>
@@ -2268,14 +2267,14 @@
       </c>
       <c r="C3" s="11">
         <f>+SUM(D3:H3)</f>
-        <v>1375</v>
-      </c>
-      <c r="D3" s="31">
-        <v>1375</v>
+        <v>1230</v>
+      </c>
+      <c r="D3" s="34">
+        <v>1230</v>
       </c>
       <c r="I3" s="26">
         <f>IFERROR(C3/6/COUNT(D3:H3),0)</f>
-        <v>229.16666666666666</v>
+        <v>205</v>
       </c>
       <c r="J3" s="3"/>
     </row>
@@ -2288,20 +2287,20 @@
       </c>
       <c r="C4" s="11">
         <f t="shared" ref="C4:C8" si="1">+SUM(D4:H4)</f>
-        <v>1092</v>
-      </c>
-      <c r="D4" s="31">
-        <v>1092</v>
+        <v>1042</v>
+      </c>
+      <c r="D4" s="34">
+        <v>1042</v>
       </c>
       <c r="I4" s="26">
         <f t="shared" ref="I4:I10" si="2">IFERROR(C4/6/COUNT(D4:H4),0)</f>
-        <v>182</v>
+        <v>173.66666666666666</v>
       </c>
       <c r="J4" s="3"/>
-      <c r="O4" s="32" t="s">
+      <c r="O4" s="31" t="s">
         <v>21</v>
       </c>
-      <c r="P4" s="32"/>
+      <c r="P4" s="31"/>
     </row>
     <row r="5" spans="1:22">
       <c r="A5" s="13" t="s">
@@ -2312,14 +2311,14 @@
       </c>
       <c r="C5" s="11">
         <f t="shared" si="1"/>
-        <v>1101</v>
-      </c>
-      <c r="D5" s="31">
-        <v>1101</v>
+        <v>1191</v>
+      </c>
+      <c r="D5" s="34">
+        <v>1191</v>
       </c>
       <c r="I5" s="26">
         <f t="shared" si="2"/>
-        <v>183.5</v>
+        <v>198.5</v>
       </c>
       <c r="J5" s="3"/>
     </row>
@@ -2332,14 +2331,14 @@
       </c>
       <c r="C6" s="11">
         <f t="shared" si="1"/>
-        <v>1178</v>
-      </c>
-      <c r="D6" s="31">
-        <v>1178</v>
+        <v>1191</v>
+      </c>
+      <c r="D6" s="34">
+        <v>1191</v>
       </c>
       <c r="I6" s="26">
         <f t="shared" si="2"/>
-        <v>196.33333333333334</v>
+        <v>198.5</v>
       </c>
       <c r="J6" s="3"/>
     </row>
@@ -2352,14 +2351,14 @@
       </c>
       <c r="C7" s="11">
         <f t="shared" si="1"/>
-        <v>1346</v>
-      </c>
-      <c r="D7" s="31">
-        <v>1346</v>
+        <v>1200</v>
+      </c>
+      <c r="D7" s="34">
+        <v>1200</v>
       </c>
       <c r="I7" s="26">
         <f t="shared" si="2"/>
-        <v>224.33333333333334</v>
+        <v>200</v>
       </c>
       <c r="J7" s="3"/>
     </row>
@@ -2372,14 +2371,14 @@
       </c>
       <c r="C8" s="11">
         <f t="shared" si="1"/>
-        <v>1310</v>
-      </c>
-      <c r="D8" s="31">
-        <v>1310</v>
+        <v>944</v>
+      </c>
+      <c r="D8" s="34">
+        <v>944</v>
       </c>
       <c r="I8" s="26">
         <f t="shared" si="2"/>
-        <v>218.33333333333334</v>
+        <v>157.33333333333334</v>
       </c>
       <c r="J8" s="3"/>
     </row>
@@ -2401,11 +2400,11 @@
       </c>
       <c r="C10" s="18">
         <f>SUM(C3:C9)</f>
-        <v>7402</v>
+        <v>6798</v>
       </c>
       <c r="D10" s="19">
         <f>SUM(D3:D9)</f>
-        <v>7402</v>
+        <v>6798</v>
       </c>
       <c r="E10" s="19">
         <f t="shared" ref="E10:H10" si="3">SUM(E3:E9)</f>
@@ -2425,7 +2424,7 @@
       </c>
       <c r="I10" s="26">
         <f t="shared" si="2"/>
-        <v>246.73333333333335</v>
+        <v>226.6</v>
       </c>
       <c r="J10" s="20"/>
       <c r="O10" s="30" t="s">
@@ -2509,25 +2508,25 @@
         <v>1</v>
       </c>
       <c r="P12" s="35">
-        <v>1375</v>
+        <v>1230</v>
       </c>
       <c r="Q12" s="35">
-        <v>1092</v>
+        <v>1042</v>
       </c>
       <c r="R12" s="35">
-        <v>1101</v>
+        <v>1191</v>
       </c>
       <c r="S12" s="35">
-        <v>1178</v>
+        <v>1191</v>
       </c>
       <c r="T12" s="35">
-        <v>1346</v>
+        <v>1200</v>
       </c>
       <c r="U12" s="35">
-        <v>1310</v>
+        <v>944</v>
       </c>
       <c r="V12" s="35">
-        <v>7402</v>
+        <v>6798</v>
       </c>
     </row>
     <row r="13" spans="1:22">
@@ -2714,25 +2713,25 @@
         <v>16</v>
       </c>
       <c r="P17" s="35">
-        <v>1375</v>
+        <v>1230</v>
       </c>
       <c r="Q17" s="35">
-        <v>1092</v>
+        <v>1042</v>
       </c>
       <c r="R17" s="35">
-        <v>1101</v>
+        <v>1191</v>
       </c>
       <c r="S17" s="35">
-        <v>1178</v>
+        <v>1191</v>
       </c>
       <c r="T17" s="35">
-        <v>1346</v>
+        <v>1200</v>
       </c>
       <c r="U17" s="35">
-        <v>1310</v>
+        <v>944</v>
       </c>
       <c r="V17" s="35">
-        <v>7402</v>
+        <v>6798</v>
       </c>
     </row>
     <row r="18" spans="1:32">
@@ -2799,8 +2798,8 @@
       <c r="J20" s="20"/>
     </row>
     <row r="21" spans="1:32">
-      <c r="A21" s="33"/>
-      <c r="B21" s="33"/>
+      <c r="A21" s="32"/>
+      <c r="B21" s="32"/>
       <c r="C21" s="2"/>
       <c r="D21" s="21"/>
       <c r="E21" s="21"/>
@@ -2809,10 +2808,10 @@
       <c r="H21" s="21"/>
       <c r="I21" s="3"/>
       <c r="J21" s="3"/>
-      <c r="O21" s="32" t="s">
+      <c r="O21" s="31" t="s">
         <v>22</v>
       </c>
-      <c r="P21" s="32"/>
+      <c r="P21" s="31"/>
     </row>
     <row r="22" spans="1:32">
       <c r="A22" s="5" t="s">
@@ -2849,7 +2848,7 @@
       </c>
       <c r="J22" s="1"/>
       <c r="O22" s="28">
-        <v>46147.854166666664</v>
+        <v>46146.854166666664</v>
       </c>
     </row>
     <row r="23" spans="1:32">
@@ -3001,8 +3000,8 @@
       <c r="J30" s="20"/>
     </row>
     <row r="31" spans="1:32">
-      <c r="A31" s="34"/>
-      <c r="B31" s="34"/>
+      <c r="A31" s="33"/>
+      <c r="B31" s="33"/>
       <c r="C31" s="3"/>
       <c r="D31" s="3"/>
       <c r="E31" s="3"/>
@@ -3235,8 +3234,8 @@
       <c r="AF40" s="27"/>
     </row>
     <row r="41" spans="1:32">
-      <c r="A41" s="34"/>
-      <c r="B41" s="34"/>
+      <c r="A41" s="33"/>
+      <c r="B41" s="33"/>
       <c r="C41" s="3"/>
       <c r="D41" s="3"/>
       <c r="E41" s="3"/>
@@ -3475,8 +3474,8 @@
       <c r="AF50" s="27"/>
     </row>
     <row r="51" spans="1:32">
-      <c r="A51" s="33"/>
-      <c r="B51" s="33"/>
+      <c r="A51" s="32"/>
+      <c r="B51" s="32"/>
       <c r="C51" s="2"/>
       <c r="D51" s="24"/>
       <c r="E51" s="24"/>
@@ -3488,8 +3487,8 @@
       <c r="AF51" s="27"/>
     </row>
     <row r="52" spans="1:32">
-      <c r="A52" s="33"/>
-      <c r="B52" s="33"/>
+      <c r="A52" s="32"/>
+      <c r="B52" s="32"/>
       <c r="C52" s="2"/>
       <c r="D52" s="21">
         <v>0</v>
@@ -3510,8 +3509,8 @@
       <c r="J52" s="3"/>
     </row>
     <row r="53" spans="1:32">
-      <c r="A53" s="33"/>
-      <c r="B53" s="33"/>
+      <c r="A53" s="32"/>
+      <c r="B53" s="32"/>
       <c r="C53" s="3"/>
       <c r="D53" s="3"/>
       <c r="E53" s="3"/>
@@ -3803,7 +3802,22 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1CB9C6E1-9ED5-4F9E-A921-9601F6BFCC2B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1CB9C6E1-9ED5-4F9E-A921-9601F6BFCC2B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="e4f8e1ef-7590-4615-a0b0-41d92864fb7e"/>
+    <ds:schemaRef ds:uri="396b9688-3d64-4f4f-b40d-59fd809f50b1"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Correccion horas y Sudoku
</commit_message>
<xml_diff>
--- a/SUDOKU.xlsx
+++ b/SUDOKU.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gplaneta.sharepoint.com/sites/BIPOWER/Shared Documents/General/Distribución Atenea/Codigos/Distribución OBS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="395" documentId="13_ncr:1_{0AD06FF4-A909-423F-B378-69C0033412ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E00A7A31-F7E6-41C9-B715-1D2F69B55449}"/>
+  <xr:revisionPtr revIDLastSave="399" documentId="13_ncr:1_{0AD06FF4-A909-423F-B378-69C0033412ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F97BD725-1B7A-4BC6-95B6-142A76792FC5}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{EF95C2B5-218E-4516-887F-CDE11964293A}"/>
   </bookViews>
@@ -17,7 +17,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="33" r:id="rId2"/>
+    <pivotCache cacheId="23" r:id="rId2"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -1486,7 +1486,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Santiago Calvo Prieto" refreshedDate="46155.771338194441" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="48" xr:uid="{93C581A5-61B5-40FF-AC76-618DD97B7B96}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Santiago Calvo Prieto" refreshedDate="46177.42890324074" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="48" xr:uid="{93C581A5-61B5-40FF-AC76-618DD97B7B96}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A2:C50" sheet="Estatus diario"/>
   </cacheSource>
@@ -1520,7 +1520,7 @@
       </sharedItems>
     </cacheField>
     <cacheField name="HS" numFmtId="0">
-      <sharedItems containsBlank="1" containsMixedTypes="1" containsNumber="1" containsInteger="1" minValue="0" maxValue="6959"/>
+      <sharedItems containsBlank="1" containsMixedTypes="1" containsNumber="1" containsInteger="1" minValue="0" maxValue="5998"/>
     </cacheField>
   </cacheFields>
   <extLst>
@@ -1536,42 +1536,42 @@
   <r>
     <x v="0"/>
     <x v="0"/>
-    <n v="1255"/>
+    <n v="907"/>
   </r>
   <r>
     <x v="0"/>
     <x v="1"/>
-    <n v="866"/>
+    <n v="862"/>
   </r>
   <r>
     <x v="0"/>
     <x v="2"/>
-    <n v="1083"/>
+    <n v="969"/>
   </r>
   <r>
     <x v="0"/>
     <x v="3"/>
-    <n v="1071"/>
+    <n v="872"/>
   </r>
   <r>
     <x v="0"/>
     <x v="4"/>
-    <n v="1020"/>
+    <n v="966"/>
   </r>
   <r>
     <x v="0"/>
     <x v="5"/>
-    <n v="848"/>
+    <n v="786"/>
   </r>
   <r>
     <x v="0"/>
     <x v="6"/>
-    <n v="816"/>
+    <n v="636"/>
   </r>
   <r>
     <x v="0"/>
     <x v="7"/>
-    <n v="6959"/>
+    <n v="5998"/>
   </r>
   <r>
     <x v="1"/>
@@ -1777,7 +1777,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{96476416-5E19-428A-9C28-862565FD05AB}" name="TablaDinámica2" cacheId="33" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{96476416-5E19-428A-9C28-862565FD05AB}" name="TablaDinámica2" cacheId="23" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="O10:W17" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="3">
     <pivotField axis="axisRow" showAll="0">
@@ -2205,9 +2205,7 @@
     <col min="14" max="14" width="5.5703125" customWidth="1"/>
     <col min="15" max="15" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="4.140625" bestFit="1" customWidth="1"/>
-    <col min="18" max="20" width="5.140625" bestFit="1" customWidth="1"/>
-    <col min="21" max="22" width="4.140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="22" width="4.140625" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="24" max="26" width="3.140625" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="3" bestFit="1" customWidth="1"/>
@@ -2276,14 +2274,14 @@
       </c>
       <c r="C3" s="11">
         <f>+SUM(D3:H3)</f>
-        <v>1255</v>
+        <v>907</v>
       </c>
       <c r="D3" s="31">
-        <v>1255</v>
+        <v>907</v>
       </c>
       <c r="I3" s="26">
         <f>IFERROR(C3/6/COUNT(D3:H3),0)</f>
-        <v>209.16666666666666</v>
+        <v>151.16666666666666</v>
       </c>
       <c r="J3" s="3"/>
     </row>
@@ -2296,14 +2294,14 @@
       </c>
       <c r="C4" s="11">
         <f t="shared" ref="C4:C9" si="1">+SUM(D4:H4)</f>
-        <v>866</v>
+        <v>862</v>
       </c>
       <c r="D4" s="31">
-        <v>866</v>
+        <v>862</v>
       </c>
       <c r="I4" s="26">
         <f t="shared" ref="I4:I10" si="2">IFERROR(C4/6/COUNT(D4:H4),0)</f>
-        <v>144.33333333333334</v>
+        <v>143.66666666666666</v>
       </c>
       <c r="J4" s="3"/>
       <c r="O4" s="32" t="s">
@@ -2320,14 +2318,14 @@
       </c>
       <c r="C5" s="11">
         <f t="shared" si="1"/>
-        <v>1083</v>
+        <v>969</v>
       </c>
       <c r="D5" s="31">
-        <v>1083</v>
+        <v>969</v>
       </c>
       <c r="I5" s="26">
         <f t="shared" si="2"/>
-        <v>180.5</v>
+        <v>161.5</v>
       </c>
       <c r="J5" s="3"/>
     </row>
@@ -2340,14 +2338,14 @@
       </c>
       <c r="C6" s="11">
         <f t="shared" si="1"/>
-        <v>1071</v>
+        <v>872</v>
       </c>
       <c r="D6" s="31">
-        <v>1071</v>
+        <v>872</v>
       </c>
       <c r="I6" s="26">
         <f t="shared" si="2"/>
-        <v>178.5</v>
+        <v>145.33333333333334</v>
       </c>
       <c r="J6" s="3"/>
     </row>
@@ -2360,14 +2358,14 @@
       </c>
       <c r="C7" s="11">
         <f t="shared" si="1"/>
-        <v>1020</v>
+        <v>966</v>
       </c>
       <c r="D7" s="31">
-        <v>1020</v>
+        <v>966</v>
       </c>
       <c r="I7" s="26">
         <f t="shared" si="2"/>
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="J7" s="3"/>
     </row>
@@ -2380,14 +2378,14 @@
       </c>
       <c r="C8" s="11">
         <f t="shared" si="1"/>
-        <v>848</v>
+        <v>786</v>
       </c>
       <c r="D8" s="31">
-        <v>848</v>
+        <v>786</v>
       </c>
       <c r="I8" s="26">
         <f t="shared" si="2"/>
-        <v>141.33333333333334</v>
+        <v>131</v>
       </c>
       <c r="J8" s="3"/>
     </row>
@@ -2400,10 +2398,10 @@
       </c>
       <c r="C9" s="11">
         <f t="shared" si="1"/>
-        <v>816</v>
+        <v>636</v>
       </c>
       <c r="D9" s="31">
-        <v>816</v>
+        <v>636</v>
       </c>
       <c r="I9" s="26"/>
       <c r="J9" s="3"/>
@@ -2417,11 +2415,11 @@
       </c>
       <c r="C10" s="18">
         <f>SUM(C3:C9)</f>
-        <v>6959</v>
+        <v>5998</v>
       </c>
       <c r="D10" s="19">
         <f>SUM(D3:D9)</f>
-        <v>6959</v>
+        <v>5998</v>
       </c>
       <c r="E10" s="19">
         <f t="shared" ref="E10:H10" si="3">SUM(E3:E9)</f>
@@ -2441,7 +2439,7 @@
       </c>
       <c r="I10" s="26">
         <f t="shared" si="2"/>
-        <v>231.96666666666664</v>
+        <v>199.93333333333334</v>
       </c>
       <c r="J10" s="20"/>
       <c r="O10" s="30" t="s">
@@ -2528,28 +2526,28 @@
         <v>1</v>
       </c>
       <c r="P12" s="35">
-        <v>1255</v>
+        <v>907</v>
       </c>
       <c r="Q12" s="35">
-        <v>866</v>
+        <v>862</v>
       </c>
       <c r="R12" s="35">
-        <v>1083</v>
+        <v>969</v>
       </c>
       <c r="S12" s="35">
-        <v>1071</v>
+        <v>872</v>
       </c>
       <c r="T12" s="35">
-        <v>1020</v>
+        <v>966</v>
       </c>
       <c r="U12" s="35">
-        <v>848</v>
+        <v>786</v>
       </c>
       <c r="V12" s="35">
-        <v>816</v>
+        <v>636</v>
       </c>
       <c r="W12" s="35">
-        <v>6959</v>
+        <v>5998</v>
       </c>
     </row>
     <row r="13" spans="1:23">
@@ -2740,28 +2738,28 @@
         <v>16</v>
       </c>
       <c r="P17" s="35">
-        <v>1255</v>
+        <v>907</v>
       </c>
       <c r="Q17" s="35">
-        <v>866</v>
+        <v>862</v>
       </c>
       <c r="R17" s="35">
-        <v>1083</v>
+        <v>969</v>
       </c>
       <c r="S17" s="35">
-        <v>1071</v>
+        <v>872</v>
       </c>
       <c r="T17" s="35">
-        <v>1020</v>
+        <v>966</v>
       </c>
       <c r="U17" s="35">
-        <v>848</v>
+        <v>786</v>
       </c>
       <c r="V17" s="35">
-        <v>816</v>
+        <v>636</v>
       </c>
       <c r="W17" s="35">
-        <v>6959</v>
+        <v>5998</v>
       </c>
     </row>
     <row r="18" spans="1:32">
@@ -2878,7 +2876,7 @@
       </c>
       <c r="J22" s="1"/>
       <c r="O22" s="28">
-        <v>46146.854166666664</v>
+        <v>46176.854166666664</v>
       </c>
     </row>
     <row r="23" spans="1:32">
@@ -3801,6 +3799,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="396b9688-3d64-4f4f-b40d-59fd809f50b1" xsi:nil="true"/>
@@ -3809,15 +3816,6 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3840,6 +3838,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{73BCA648-DFB0-4933-AD78-DBDD8CAF7C52}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{007506E0-0CDE-4051-B6C4-9C0A8A8B90A4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -3848,12 +3854,4 @@
     <ds:schemaRef ds:uri="e4f8e1ef-7590-4615-a0b0-41d92864fb7e"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{73BCA648-DFB0-4933-AD78-DBDD8CAF7C52}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Correcciones conteo de cupones. Filtros PILAR
</commit_message>
<xml_diff>
--- a/SUDOKU.xlsx
+++ b/SUDOKU.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gplaneta.sharepoint.com/sites/BIPOWER/Shared Documents/General/Distribución Atenea/Codigos/Distribución OBS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="399" documentId="13_ncr:1_{0AD06FF4-A909-423F-B378-69C0033412ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F97BD725-1B7A-4BC6-95B6-142A76792FC5}"/>
+  <xr:revisionPtr revIDLastSave="403" documentId="13_ncr:1_{0AD06FF4-A909-423F-B378-69C0033412ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DF10FCB0-2A55-4AEA-80FA-03647C972CAD}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{EF95C2B5-218E-4516-887F-CDE11964293A}"/>
   </bookViews>
@@ -17,7 +17,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="23" r:id="rId2"/>
+    <pivotCache cacheId="18" r:id="rId2"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -1486,7 +1486,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Santiago Calvo Prieto" refreshedDate="46177.42890324074" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="48" xr:uid="{93C581A5-61B5-40FF-AC76-618DD97B7B96}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Santiago Calvo Prieto" refreshedDate="46209.515215740743" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="48" xr:uid="{93C581A5-61B5-40FF-AC76-618DD97B7B96}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A2:C50" sheet="Estatus diario"/>
   </cacheSource>
@@ -1520,7 +1520,7 @@
       </sharedItems>
     </cacheField>
     <cacheField name="HS" numFmtId="0">
-      <sharedItems containsBlank="1" containsMixedTypes="1" containsNumber="1" containsInteger="1" minValue="0" maxValue="5998"/>
+      <sharedItems containsBlank="1" containsMixedTypes="1" containsNumber="1" containsInteger="1" minValue="0" maxValue="8556"/>
     </cacheField>
   </cacheFields>
   <extLst>
@@ -1536,42 +1536,42 @@
   <r>
     <x v="0"/>
     <x v="0"/>
-    <n v="907"/>
+    <n v="1250"/>
   </r>
   <r>
     <x v="0"/>
     <x v="1"/>
-    <n v="862"/>
+    <n v="1160"/>
   </r>
   <r>
     <x v="0"/>
     <x v="2"/>
-    <n v="969"/>
+    <n v="1456"/>
   </r>
   <r>
     <x v="0"/>
     <x v="3"/>
-    <n v="872"/>
+    <n v="1280"/>
   </r>
   <r>
     <x v="0"/>
     <x v="4"/>
-    <n v="966"/>
+    <n v="1320"/>
   </r>
   <r>
     <x v="0"/>
     <x v="5"/>
-    <n v="786"/>
+    <n v="1254"/>
   </r>
   <r>
     <x v="0"/>
     <x v="6"/>
-    <n v="636"/>
+    <n v="836"/>
   </r>
   <r>
     <x v="0"/>
     <x v="7"/>
-    <n v="5998"/>
+    <n v="8556"/>
   </r>
   <r>
     <x v="1"/>
@@ -1777,7 +1777,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{96476416-5E19-428A-9C28-862565FD05AB}" name="TablaDinámica2" cacheId="23" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{96476416-5E19-428A-9C28-862565FD05AB}" name="TablaDinámica2" cacheId="18" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="O10:W17" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="3">
     <pivotField axis="axisRow" showAll="0">
@@ -2205,7 +2205,8 @@
     <col min="14" max="14" width="5.5703125" customWidth="1"/>
     <col min="15" max="15" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="17" max="22" width="4.140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="21" width="5.140625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="4.140625" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="24" max="26" width="3.140625" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="3" bestFit="1" customWidth="1"/>
@@ -2274,14 +2275,14 @@
       </c>
       <c r="C3" s="11">
         <f>+SUM(D3:H3)</f>
-        <v>907</v>
+        <v>1250</v>
       </c>
       <c r="D3" s="31">
-        <v>907</v>
+        <v>1250</v>
       </c>
       <c r="I3" s="26">
         <f>IFERROR(C3/6/COUNT(D3:H3),0)</f>
-        <v>151.16666666666666</v>
+        <v>208.33333333333334</v>
       </c>
       <c r="J3" s="3"/>
     </row>
@@ -2294,14 +2295,14 @@
       </c>
       <c r="C4" s="11">
         <f t="shared" ref="C4:C9" si="1">+SUM(D4:H4)</f>
-        <v>862</v>
+        <v>1160</v>
       </c>
       <c r="D4" s="31">
-        <v>862</v>
+        <v>1160</v>
       </c>
       <c r="I4" s="26">
         <f t="shared" ref="I4:I10" si="2">IFERROR(C4/6/COUNT(D4:H4),0)</f>
-        <v>143.66666666666666</v>
+        <v>193.33333333333334</v>
       </c>
       <c r="J4" s="3"/>
       <c r="O4" s="32" t="s">
@@ -2318,14 +2319,14 @@
       </c>
       <c r="C5" s="11">
         <f t="shared" si="1"/>
-        <v>969</v>
+        <v>1456</v>
       </c>
       <c r="D5" s="31">
-        <v>969</v>
+        <v>1456</v>
       </c>
       <c r="I5" s="26">
         <f t="shared" si="2"/>
-        <v>161.5</v>
+        <v>242.66666666666666</v>
       </c>
       <c r="J5" s="3"/>
     </row>
@@ -2338,14 +2339,14 @@
       </c>
       <c r="C6" s="11">
         <f t="shared" si="1"/>
-        <v>872</v>
+        <v>1280</v>
       </c>
       <c r="D6" s="31">
-        <v>872</v>
+        <v>1280</v>
       </c>
       <c r="I6" s="26">
         <f t="shared" si="2"/>
-        <v>145.33333333333334</v>
+        <v>213.33333333333334</v>
       </c>
       <c r="J6" s="3"/>
     </row>
@@ -2358,14 +2359,14 @@
       </c>
       <c r="C7" s="11">
         <f t="shared" si="1"/>
-        <v>966</v>
+        <v>1320</v>
       </c>
       <c r="D7" s="31">
-        <v>966</v>
+        <v>1320</v>
       </c>
       <c r="I7" s="26">
         <f t="shared" si="2"/>
-        <v>161</v>
+        <v>220</v>
       </c>
       <c r="J7" s="3"/>
     </row>
@@ -2378,14 +2379,14 @@
       </c>
       <c r="C8" s="11">
         <f t="shared" si="1"/>
-        <v>786</v>
+        <v>1254</v>
       </c>
       <c r="D8" s="31">
-        <v>786</v>
+        <v>1254</v>
       </c>
       <c r="I8" s="26">
         <f t="shared" si="2"/>
-        <v>131</v>
+        <v>209</v>
       </c>
       <c r="J8" s="3"/>
     </row>
@@ -2398,10 +2399,10 @@
       </c>
       <c r="C9" s="11">
         <f t="shared" si="1"/>
-        <v>636</v>
+        <v>836</v>
       </c>
       <c r="D9" s="31">
-        <v>636</v>
+        <v>836</v>
       </c>
       <c r="I9" s="26"/>
       <c r="J9" s="3"/>
@@ -2415,11 +2416,11 @@
       </c>
       <c r="C10" s="18">
         <f>SUM(C3:C9)</f>
-        <v>5998</v>
+        <v>8556</v>
       </c>
       <c r="D10" s="19">
         <f>SUM(D3:D9)</f>
-        <v>5998</v>
+        <v>8556</v>
       </c>
       <c r="E10" s="19">
         <f t="shared" ref="E10:H10" si="3">SUM(E3:E9)</f>
@@ -2439,7 +2440,7 @@
       </c>
       <c r="I10" s="26">
         <f t="shared" si="2"/>
-        <v>199.93333333333334</v>
+        <v>285.2</v>
       </c>
       <c r="J10" s="20"/>
       <c r="O10" s="30" t="s">
@@ -2526,28 +2527,28 @@
         <v>1</v>
       </c>
       <c r="P12" s="35">
-        <v>907</v>
+        <v>1250</v>
       </c>
       <c r="Q12" s="35">
-        <v>862</v>
+        <v>1160</v>
       </c>
       <c r="R12" s="35">
-        <v>969</v>
+        <v>1456</v>
       </c>
       <c r="S12" s="35">
-        <v>872</v>
+        <v>1280</v>
       </c>
       <c r="T12" s="35">
-        <v>966</v>
+        <v>1320</v>
       </c>
       <c r="U12" s="35">
-        <v>786</v>
+        <v>1254</v>
       </c>
       <c r="V12" s="35">
-        <v>636</v>
+        <v>836</v>
       </c>
       <c r="W12" s="35">
-        <v>5998</v>
+        <v>8556</v>
       </c>
     </row>
     <row r="13" spans="1:23">
@@ -2738,28 +2739,28 @@
         <v>16</v>
       </c>
       <c r="P17" s="35">
-        <v>907</v>
+        <v>1250</v>
       </c>
       <c r="Q17" s="35">
-        <v>862</v>
+        <v>1160</v>
       </c>
       <c r="R17" s="35">
-        <v>969</v>
+        <v>1456</v>
       </c>
       <c r="S17" s="35">
-        <v>872</v>
+        <v>1280</v>
       </c>
       <c r="T17" s="35">
-        <v>966</v>
+        <v>1320</v>
       </c>
       <c r="U17" s="35">
-        <v>786</v>
+        <v>1254</v>
       </c>
       <c r="V17" s="35">
-        <v>636</v>
+        <v>836</v>
       </c>
       <c r="W17" s="35">
-        <v>5998</v>
+        <v>8556</v>
       </c>
     </row>
     <row r="18" spans="1:32">

</xml_diff>